<commit_message>
Fase  1 2 y 3 listo
</commit_message>
<xml_diff>
--- a/Reestructuracion_Expandido.xlsx
+++ b/Reestructuracion_Expandido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\www\validador-deis-sso\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67E067BD-491D-4A97-B74E-26EA6211FC8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B39A955-6B03-4A5E-B54E-DD2F1652808D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$M$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$M$130</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1420" uniqueCount="502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1420" uniqueCount="507">
   <si>
     <t>ID</t>
   </si>
@@ -1240,9 +1240,6 @@
     <t>P2</t>
   </si>
   <si>
-    <t>SECCIÓN A</t>
-  </si>
-  <si>
     <t>Población en Control, suma de C12 menos F12 y G12</t>
   </si>
   <si>
@@ -1378,9 +1375,6 @@
     <t>C17</t>
   </si>
   <si>
-    <t>SECCIÓN B</t>
-  </si>
-  <si>
     <t>Metas de Compensación Hba1C&lt; 7%</t>
   </si>
   <si>
@@ -1420,24 +1414,15 @@
     <t>FILA 38</t>
   </si>
   <si>
-    <t>SECCIÓN A1</t>
-  </si>
-  <si>
     <t>Programa Más Adultos Mayores Autovalentes</t>
   </si>
   <si>
     <t>C29+D29</t>
   </si>
   <si>
-    <t>PMAA</t>
-  </si>
-  <si>
     <t>P6</t>
   </si>
   <si>
-    <t>SECCIÓN A.1</t>
-  </si>
-  <si>
     <t>Población en control al corte, personas con diagnóstico de trastorno mentales</t>
   </si>
   <si>
@@ -1453,9 +1438,6 @@
     <t>SUM(C25:C58)</t>
   </si>
   <si>
-    <t>SECCIÓN B.1</t>
-  </si>
-  <si>
     <t>C86</t>
   </si>
   <si>
@@ -1525,9 +1507,6 @@
     <t>SUM(B12:B19)</t>
   </si>
   <si>
-    <t>TODOS EXCEPTO HPU, HRN</t>
-  </si>
-  <si>
     <t xml:space="preserve">SECCION B: GESTANTES EN CONTROL CON EVALUACIÓN RIESGO BIOPSICOSOCIAL </t>
   </si>
   <si>
@@ -1540,15 +1519,6 @@
     <t>SECCION C: GESTANTES EN RIESGO PSICOSOCIAL CON VISITA DOMICILIARIA INTEGRAL REALIZADA EN EL SEMESTRE</t>
   </si>
   <si>
-    <t>SECCIÓN D</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> SECCIÓN D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SECCIÓN A </t>
-  </si>
-  <si>
     <t>SECCION D: GESTANTES Y PERSONAS DE 8° MES POST-PARTO EN CONTROL, SEGÚN ESTADO NUTRICIONALL</t>
   </si>
   <si>
@@ -1565,6 +1535,51 @@
   </si>
   <si>
     <t>C12+ (F12-G12)</t>
+  </si>
+  <si>
+    <t>SECCIÓN A: EXISTENCIA DE POBLACIÓN EN CONTROL</t>
+  </si>
+  <si>
+    <t>SECCION D: NIVEL DE CONTROL DE POBLACION RESPIRATORIA CRONICA</t>
+  </si>
+  <si>
+    <t>SECCIÓN A: PROGRAMA SALUD CARDIOVASCULAR (PSCV)</t>
+  </si>
+  <si>
+    <t>SECCIÓN B: METAS DE COMPENSACIÓN</t>
+  </si>
+  <si>
+    <t>SECCION A: POBLACIÓN EN CONTROL POR CONDICIÓN DE FUNCIONALIDAD</t>
+  </si>
+  <si>
+    <t>SECCION A.1: EXISTENCIA DE POBLACIÓN EN CONTROL EN PROGRAMA "MÁS ADULTOS MAYORES AUTOVALENTES" POR CONDICIÓN DE FUNCIONALIDAD</t>
+  </si>
+  <si>
+    <t>SECCION B: POBLACIÓN BAJO CONTROL POR ESTADO NUTRICIONAL</t>
+  </si>
+  <si>
+    <t>SECCION A.1: POBLACIÓN EN CONTROL EN APS AL CORTE</t>
+  </si>
+  <si>
+    <t>SECCION B.1: POBLACIÓN EN CONTROL EN ESPECIALIDAD AL CORTE</t>
+  </si>
+  <si>
+    <t>SECCIÓN A. CLASIFICACIÓN DE LAS FAMILIAS SECTOR URBANO</t>
+  </si>
+  <si>
+    <t>SECCIÓN A.1 CLASIFICACIÓN DE LAS FAMILIAS SECTOR RURAL</t>
+  </si>
+  <si>
+    <t>SECCION A: POBLACIÓN EN CONTROL DEL PROGRAMA DE VIH/SIDA</t>
+  </si>
+  <si>
+    <t>SECCION B: POBLACIÓN EN CONTROL POR COMERCIO SEXUAL</t>
+  </si>
+  <si>
+    <t>SECCIÓN A: PROGRAMA DE CANCER DE CUELLO UTERINO</t>
+  </si>
+  <si>
+    <t>CESFAM</t>
   </si>
 </sst>
 </file>
@@ -1720,21 +1735,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF00B050"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <b/>
@@ -5407,10 +5408,10 @@
         <v>362</v>
       </c>
       <c r="E94" s="10" t="s">
-        <v>490</v>
+        <v>483</v>
       </c>
       <c r="F94" s="11" t="s">
-        <v>491</v>
+        <v>484</v>
       </c>
       <c r="G94" s="11" t="s">
         <v>363</v>
@@ -5422,7 +5423,7 @@
         <v>362</v>
       </c>
       <c r="J94" s="10" t="s">
-        <v>489</v>
+        <v>482</v>
       </c>
       <c r="K94" s="11" t="s">
         <v>364</v>
@@ -5448,7 +5449,7 @@
         <v>362</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>492</v>
+        <v>485</v>
       </c>
       <c r="F95" s="11" t="s">
         <v>366</v>
@@ -5489,7 +5490,7 @@
         <v>362</v>
       </c>
       <c r="E96" s="10" t="s">
-        <v>496</v>
+        <v>486</v>
       </c>
       <c r="F96" s="11" t="s">
         <v>368</v>
@@ -5504,7 +5505,7 @@
         <v>362</v>
       </c>
       <c r="J96" s="10" t="s">
-        <v>498</v>
+        <v>488</v>
       </c>
       <c r="K96" s="11" t="s">
         <v>370</v>
@@ -5530,7 +5531,7 @@
         <v>362</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>490</v>
+        <v>483</v>
       </c>
       <c r="F97" s="11" t="s">
         <v>371</v>
@@ -5545,7 +5546,7 @@
         <v>362</v>
       </c>
       <c r="J97" s="10" t="s">
-        <v>498</v>
+        <v>488</v>
       </c>
       <c r="K97" s="11" t="s">
         <v>373</v>
@@ -5571,7 +5572,7 @@
         <v>362</v>
       </c>
       <c r="E98" s="10" t="s">
-        <v>490</v>
+        <v>483</v>
       </c>
       <c r="F98" s="11" t="s">
         <v>375</v>
@@ -5586,7 +5587,7 @@
         <v>362</v>
       </c>
       <c r="J98" s="10" t="s">
-        <v>498</v>
+        <v>488</v>
       </c>
       <c r="K98" s="11" t="s">
         <v>377</v>
@@ -5612,7 +5613,7 @@
         <v>362</v>
       </c>
       <c r="E99" s="10" t="s">
-        <v>497</v>
+        <v>487</v>
       </c>
       <c r="F99" s="11" t="s">
         <v>379</v>
@@ -5627,7 +5628,7 @@
         <v>362</v>
       </c>
       <c r="J99" s="10" t="s">
-        <v>497</v>
+        <v>487</v>
       </c>
       <c r="K99" s="11" t="s">
         <v>381</v>
@@ -5653,7 +5654,7 @@
         <v>362</v>
       </c>
       <c r="E100" s="10" t="s">
-        <v>497</v>
+        <v>487</v>
       </c>
       <c r="F100" s="11" t="s">
         <v>383</v>
@@ -5668,7 +5669,7 @@
         <v>362</v>
       </c>
       <c r="J100" s="10" t="s">
-        <v>497</v>
+        <v>487</v>
       </c>
       <c r="K100" s="11" t="s">
         <v>385</v>
@@ -5694,7 +5695,7 @@
         <v>362</v>
       </c>
       <c r="E101" s="10" t="s">
-        <v>497</v>
+        <v>487</v>
       </c>
       <c r="F101" s="11" t="s">
         <v>387</v>
@@ -5709,7 +5710,7 @@
         <v>362</v>
       </c>
       <c r="J101" s="10" t="s">
-        <v>497</v>
+        <v>487</v>
       </c>
       <c r="K101" s="11" t="s">
         <v>388</v>
@@ -5735,7 +5736,7 @@
         <v>362</v>
       </c>
       <c r="E102" s="10" t="s">
-        <v>499</v>
+        <v>489</v>
       </c>
       <c r="F102" s="11" t="s">
         <v>390</v>
@@ -5776,13 +5777,13 @@
         <v>392</v>
       </c>
       <c r="E103" s="16" t="s">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>501</v>
+        <v>491</v>
       </c>
       <c r="H103" s="2" t="s">
         <v>231</v>
@@ -5791,13 +5792,13 @@
         <v>392</v>
       </c>
       <c r="J103" s="16" t="s">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="K103" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="L103" s="1" t="s">
         <v>395</v>
-      </c>
-      <c r="L103" s="1" t="s">
-        <v>396</v>
       </c>
       <c r="M103" s="1" t="s">
         <v>19</v>
@@ -5817,10 +5818,10 @@
         <v>392</v>
       </c>
       <c r="E104" s="16" t="s">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="G104" s="2" t="s">
         <v>35</v>
@@ -5832,13 +5833,13 @@
         <v>392</v>
       </c>
       <c r="J104" s="16" t="s">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="K104" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="L104" s="1" t="s">
         <v>398</v>
-      </c>
-      <c r="L104" s="1" t="s">
-        <v>399</v>
       </c>
       <c r="M104" s="1" t="s">
         <v>19</v>
@@ -5858,13 +5859,13 @@
         <v>392</v>
       </c>
       <c r="E105" s="16" t="s">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="F105" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="G105" s="2" t="s">
         <v>400</v>
-      </c>
-      <c r="G105" s="2" t="s">
-        <v>401</v>
       </c>
       <c r="H105" s="2" t="s">
         <v>231</v>
@@ -5873,13 +5874,13 @@
         <v>392</v>
       </c>
       <c r="J105" s="16" t="s">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="K105" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="L105" s="1" t="s">
         <v>402</v>
-      </c>
-      <c r="L105" s="1" t="s">
-        <v>403</v>
       </c>
       <c r="M105" s="1" t="s">
         <v>19</v>
@@ -5899,13 +5900,13 @@
         <v>392</v>
       </c>
       <c r="E106" s="16" t="s">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="F106" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="G106" s="2" t="s">
         <v>404</v>
-      </c>
-      <c r="G106" s="2" t="s">
-        <v>405</v>
       </c>
       <c r="H106" s="2" t="s">
         <v>231</v>
@@ -5914,13 +5915,13 @@
         <v>392</v>
       </c>
       <c r="J106" s="16" t="s">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="K106" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="L106" s="1" t="s">
         <v>406</v>
-      </c>
-      <c r="L106" s="1" t="s">
-        <v>407</v>
       </c>
       <c r="M106" s="1" t="s">
         <v>19</v>
@@ -5937,37 +5938,37 @@
         <v>14</v>
       </c>
       <c r="D107" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="E107" s="16" t="s">
+        <v>492</v>
+      </c>
+      <c r="F107" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="E107" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="F107" s="2" t="s">
+      <c r="G107" s="2" t="s">
         <v>409</v>
-      </c>
-      <c r="G107" s="2" t="s">
-        <v>410</v>
       </c>
       <c r="H107" s="2" t="s">
         <v>294</v>
       </c>
       <c r="I107" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="J107" s="2" t="s">
-        <v>393</v>
+        <v>407</v>
+      </c>
+      <c r="J107" s="16" t="s">
+        <v>492</v>
       </c>
       <c r="K107" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="L107" s="1" t="s">
         <v>411</v>
       </c>
-      <c r="L107" s="1" t="s">
-        <v>412</v>
-      </c>
       <c r="M107" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>242</v>
       </c>
@@ -5978,31 +5979,31 @@
         <v>14</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>408</v>
-      </c>
-      <c r="E108" s="2" t="s">
-        <v>393</v>
+        <v>407</v>
+      </c>
+      <c r="E108" s="16" t="s">
+        <v>492</v>
       </c>
       <c r="F108" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="G108" s="2" t="s">
         <v>413</v>
-      </c>
-      <c r="G108" s="2" t="s">
-        <v>414</v>
       </c>
       <c r="H108" s="2" t="s">
         <v>294</v>
       </c>
       <c r="I108" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="J108" s="16" t="s">
+        <v>492</v>
+      </c>
+      <c r="K108" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="J108" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="K108" s="2" t="s">
+      <c r="L108" s="1" t="s">
         <v>409</v>
-      </c>
-      <c r="L108" s="1" t="s">
-        <v>410</v>
       </c>
       <c r="M108" s="1" t="s">
         <v>19</v>
@@ -6019,31 +6020,31 @@
         <v>14</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>408</v>
-      </c>
-      <c r="E109" s="2" t="s">
-        <v>393</v>
+        <v>407</v>
+      </c>
+      <c r="E109" s="16" t="s">
+        <v>492</v>
       </c>
       <c r="F109" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="G109" s="2" t="s">
         <v>415</v>
-      </c>
-      <c r="G109" s="2" t="s">
-        <v>416</v>
       </c>
       <c r="H109" s="2" t="s">
         <v>231</v>
       </c>
       <c r="I109" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="J109" s="2" t="s">
-        <v>494</v>
+        <v>407</v>
+      </c>
+      <c r="J109" s="16" t="s">
+        <v>493</v>
       </c>
       <c r="K109" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="L109" s="1" t="s">
         <v>417</v>
-      </c>
-      <c r="L109" s="1" t="s">
-        <v>418</v>
       </c>
       <c r="M109" s="1" t="s">
         <v>19</v>
@@ -6060,31 +6061,31 @@
         <v>14</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>408</v>
-      </c>
-      <c r="E110" s="2" t="s">
-        <v>393</v>
+        <v>407</v>
+      </c>
+      <c r="E110" s="16" t="s">
+        <v>492</v>
       </c>
       <c r="F110" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G110" s="2" t="s">
         <v>419</v>
-      </c>
-      <c r="G110" s="2" t="s">
-        <v>420</v>
       </c>
       <c r="H110" s="2" t="s">
         <v>231</v>
       </c>
       <c r="I110" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="J110" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="J110" s="16" t="s">
         <v>493</v>
       </c>
       <c r="K110" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="L110" s="1" t="s">
         <v>421</v>
-      </c>
-      <c r="L110" s="1" t="s">
-        <v>422</v>
       </c>
       <c r="M110" s="1" t="s">
         <v>19</v>
@@ -6101,31 +6102,31 @@
         <v>14</v>
       </c>
       <c r="D111" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="E111" s="16" t="s">
+        <v>494</v>
+      </c>
+      <c r="F111" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="E111" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="F111" s="2" t="s">
+      <c r="G111" s="2" t="s">
         <v>424</v>
-      </c>
-      <c r="G111" s="2" t="s">
-        <v>425</v>
       </c>
       <c r="H111" s="2" t="s">
         <v>294</v>
       </c>
       <c r="I111" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="J111" s="2" t="s">
-        <v>393</v>
+        <v>422</v>
+      </c>
+      <c r="J111" s="16" t="s">
+        <v>494</v>
       </c>
       <c r="K111" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="L111" s="1" t="s">
         <v>426</v>
-      </c>
-      <c r="L111" s="1" t="s">
-        <v>427</v>
       </c>
       <c r="M111" s="1" t="s">
         <v>19</v>
@@ -6142,37 +6143,37 @@
         <v>14</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>423</v>
-      </c>
-      <c r="E112" s="2" t="s">
-        <v>393</v>
+        <v>422</v>
+      </c>
+      <c r="E112" s="16" t="s">
+        <v>494</v>
       </c>
       <c r="F112" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="G112" s="2" t="s">
         <v>428</v>
-      </c>
-      <c r="G112" s="2" t="s">
-        <v>429</v>
       </c>
       <c r="H112" s="2" t="s">
         <v>294</v>
       </c>
       <c r="I112" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="J112" s="2" t="s">
-        <v>439</v>
+        <v>422</v>
+      </c>
+      <c r="J112" s="16" t="s">
+        <v>495</v>
       </c>
       <c r="K112" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="L112" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="L112" s="1" t="s">
-        <v>431</v>
-      </c>
       <c r="M112" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>242</v>
       </c>
@@ -6183,31 +6184,31 @@
         <v>14</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>423</v>
-      </c>
-      <c r="E113" s="2" t="s">
-        <v>495</v>
+        <v>422</v>
+      </c>
+      <c r="E113" s="16" t="s">
+        <v>494</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="G113" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="H113" s="2" t="s">
         <v>294</v>
       </c>
       <c r="I113" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="J113" s="2" t="s">
-        <v>439</v>
+        <v>422</v>
+      </c>
+      <c r="J113" s="16" t="s">
+        <v>495</v>
       </c>
       <c r="K113" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="L113" s="1" t="s">
         <v>433</v>
-      </c>
-      <c r="L113" s="1" t="s">
-        <v>434</v>
       </c>
       <c r="M113" s="1" t="s">
         <v>19</v>
@@ -6224,31 +6225,31 @@
         <v>14</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>423</v>
-      </c>
-      <c r="E114" s="2" t="s">
-        <v>495</v>
+        <v>422</v>
+      </c>
+      <c r="E114" s="16" t="s">
+        <v>494</v>
       </c>
       <c r="F114" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="G114" s="2" t="s">
         <v>435</v>
-      </c>
-      <c r="G114" s="2" t="s">
-        <v>436</v>
       </c>
       <c r="H114" s="2" t="s">
         <v>294</v>
       </c>
       <c r="I114" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="J114" s="2" t="s">
-        <v>439</v>
+        <v>422</v>
+      </c>
+      <c r="J114" s="16" t="s">
+        <v>495</v>
       </c>
       <c r="K114" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="L114" s="1" t="s">
         <v>437</v>
-      </c>
-      <c r="L114" s="1" t="s">
-        <v>438</v>
       </c>
       <c r="M114" s="1" t="s">
         <v>19</v>
@@ -6265,28 +6266,28 @@
         <v>14</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>423</v>
-      </c>
-      <c r="E115" s="2" t="s">
-        <v>439</v>
+        <v>422</v>
+      </c>
+      <c r="E115" s="16" t="s">
+        <v>495</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="G115" s="2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="H115" s="2" t="s">
         <v>232</v>
       </c>
       <c r="I115" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="J115" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="J115" s="16" t="s">
+        <v>495</v>
+      </c>
+      <c r="K115" s="2" t="s">
         <v>439</v>
-      </c>
-      <c r="K115" s="2" t="s">
-        <v>441</v>
       </c>
       <c r="L115" s="1" t="s">
         <v>115</v>
@@ -6295,7 +6296,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="116" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>242</v>
       </c>
@@ -6306,37 +6307,37 @@
         <v>14</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>423</v>
-      </c>
-      <c r="E116" s="2" t="s">
-        <v>495</v>
+        <v>422</v>
+      </c>
+      <c r="E116" s="16" t="s">
+        <v>494</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="G116" s="2" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="H116" s="2" t="s">
         <v>294</v>
       </c>
       <c r="I116" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="J116" s="2" t="s">
-        <v>439</v>
+        <v>422</v>
+      </c>
+      <c r="J116" s="16" t="s">
+        <v>495</v>
       </c>
       <c r="K116" s="2" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="L116" s="1" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="M116" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>242</v>
       </c>
@@ -6347,37 +6348,37 @@
         <v>14</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>423</v>
-      </c>
-      <c r="E117" s="2" t="s">
-        <v>495</v>
+        <v>422</v>
+      </c>
+      <c r="E117" s="16" t="s">
+        <v>494</v>
       </c>
       <c r="F117" s="2" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="G117" s="2" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="H117" s="2" t="s">
         <v>294</v>
       </c>
       <c r="I117" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="J117" s="2" t="s">
-        <v>439</v>
+        <v>422</v>
+      </c>
+      <c r="J117" s="16" t="s">
+        <v>495</v>
       </c>
       <c r="K117" s="2" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="L117" s="1" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="M117" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>242</v>
       </c>
@@ -6388,37 +6389,37 @@
         <v>14</v>
       </c>
       <c r="D118" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="E118" s="16" t="s">
+        <v>496</v>
+      </c>
+      <c r="F118" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="G118" s="2" t="s">
         <v>448</v>
-      </c>
-      <c r="E118" s="2" t="s">
-        <v>495</v>
-      </c>
-      <c r="F118" s="2" t="s">
-        <v>449</v>
-      </c>
-      <c r="G118" s="2" t="s">
-        <v>450</v>
       </c>
       <c r="H118" s="2" t="s">
         <v>231</v>
       </c>
       <c r="I118" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="J118" s="2" t="s">
-        <v>439</v>
+        <v>446</v>
+      </c>
+      <c r="J118" s="16" t="s">
+        <v>498</v>
       </c>
       <c r="K118" s="2" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="L118" s="1" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="M118" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="119" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>188</v>
       </c>
@@ -6429,16 +6430,16 @@
         <v>14</v>
       </c>
       <c r="D119" s="1" t="s">
-        <v>448</v>
-      </c>
-      <c r="E119" s="2" t="s">
-        <v>453</v>
+        <v>446</v>
+      </c>
+      <c r="E119" s="16" t="s">
+        <v>497</v>
       </c>
       <c r="F119" s="2" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="G119" s="2" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="H119" s="2" t="s">
         <v>230</v>
@@ -6456,7 +6457,7 @@
         <v>361</v>
       </c>
       <c r="M119" s="1" t="s">
-        <v>456</v>
+        <v>506</v>
       </c>
     </row>
     <row r="120" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -6470,13 +6471,13 @@
         <v>14</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="E120" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
+      </c>
+      <c r="E120" s="16" t="s">
+        <v>499</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>459</v>
+        <v>454</v>
       </c>
       <c r="G120" s="2" t="s">
         <v>53</v>
@@ -6485,13 +6486,13 @@
         <v>294</v>
       </c>
       <c r="I120" s="2" t="s">
-        <v>457</v>
-      </c>
-      <c r="J120" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
+      </c>
+      <c r="J120" s="16" t="s">
+        <v>499</v>
       </c>
       <c r="K120" s="2" t="s">
-        <v>460</v>
+        <v>455</v>
       </c>
       <c r="L120" s="1" t="s">
         <v>44</v>
@@ -6500,7 +6501,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>219</v>
       </c>
@@ -6511,13 +6512,13 @@
         <v>14</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="E121" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
+      </c>
+      <c r="E121" s="16" t="s">
+        <v>499</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>461</v>
+        <v>456</v>
       </c>
       <c r="G121" s="2" t="s">
         <v>53</v>
@@ -6526,16 +6527,16 @@
         <v>294</v>
       </c>
       <c r="I121" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="J121" s="16" t="s">
+        <v>499</v>
+      </c>
+      <c r="K121" s="2" t="s">
         <v>457</v>
       </c>
-      <c r="J121" s="2" t="s">
+      <c r="L121" s="1" t="s">
         <v>458</v>
-      </c>
-      <c r="K121" s="2" t="s">
-        <v>462</v>
-      </c>
-      <c r="L121" s="1" t="s">
-        <v>463</v>
       </c>
       <c r="M121" s="1" t="s">
         <v>19</v>
@@ -6552,37 +6553,37 @@
         <v>14</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="E122" s="2" t="s">
-        <v>464</v>
+        <v>453</v>
+      </c>
+      <c r="E122" s="16" t="s">
+        <v>500</v>
       </c>
       <c r="F122" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="G122" s="2" t="s">
         <v>459</v>
-      </c>
-      <c r="G122" s="2" t="s">
-        <v>465</v>
       </c>
       <c r="H122" s="2" t="s">
         <v>294</v>
       </c>
       <c r="I122" s="2" t="s">
-        <v>457</v>
-      </c>
-      <c r="J122" s="2" t="s">
-        <v>464</v>
+        <v>453</v>
+      </c>
+      <c r="J122" s="16" t="s">
+        <v>500</v>
       </c>
       <c r="K122" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="L122" s="1" t="s">
         <v>460</v>
       </c>
-      <c r="L122" s="1" t="s">
-        <v>466</v>
-      </c>
       <c r="M122" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="123" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>219</v>
       </c>
@@ -6593,31 +6594,31 @@
         <v>14</v>
       </c>
       <c r="D123" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="E123" s="2" t="s">
-        <v>464</v>
+        <v>453</v>
+      </c>
+      <c r="E123" s="16" t="s">
+        <v>500</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>467</v>
+        <v>461</v>
       </c>
       <c r="G123" s="2" t="s">
-        <v>466</v>
+        <v>460</v>
       </c>
       <c r="H123" s="2" t="s">
         <v>294</v>
       </c>
       <c r="I123" s="2" t="s">
-        <v>457</v>
-      </c>
-      <c r="J123" s="2" t="s">
-        <v>464</v>
+        <v>453</v>
+      </c>
+      <c r="J123" s="16" t="s">
+        <v>500</v>
       </c>
       <c r="K123" s="2" t="s">
-        <v>468</v>
+        <v>462</v>
       </c>
       <c r="L123" s="1" t="s">
-        <v>469</v>
+        <v>463</v>
       </c>
       <c r="M123" s="1" t="s">
         <v>19</v>
@@ -6634,28 +6635,28 @@
         <v>14</v>
       </c>
       <c r="D124" s="1" t="s">
-        <v>470</v>
-      </c>
-      <c r="E124" s="2" t="s">
-        <v>393</v>
+        <v>464</v>
+      </c>
+      <c r="E124" s="16" t="s">
+        <v>501</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="G124" s="2" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="H124" s="2" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
       <c r="I124" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="J124" s="2" t="s">
-        <v>393</v>
+        <v>464</v>
+      </c>
+      <c r="J124" s="16" t="s">
+        <v>501</v>
       </c>
       <c r="K124" s="2" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="L124" s="1" t="s">
         <v>30</v>
@@ -6675,31 +6676,31 @@
         <v>14</v>
       </c>
       <c r="D125" s="1" t="s">
-        <v>470</v>
-      </c>
-      <c r="E125" s="2" t="s">
-        <v>393</v>
+        <v>464</v>
+      </c>
+      <c r="E125" s="16" t="s">
+        <v>501</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="G125" s="2" t="s">
         <v>30</v>
       </c>
       <c r="H125" s="2" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
       <c r="I125" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="J125" s="16" t="s">
+        <v>501</v>
+      </c>
+      <c r="K125" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="L125" s="1" t="s">
         <v>470</v>
-      </c>
-      <c r="J125" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="K125" s="2" t="s">
-        <v>475</v>
-      </c>
-      <c r="L125" s="1" t="s">
-        <v>476</v>
       </c>
       <c r="M125" s="1" t="s">
         <v>19</v>
@@ -6716,31 +6717,31 @@
         <v>14</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>470</v>
-      </c>
-      <c r="E126" s="2" t="s">
-        <v>458</v>
+        <v>464</v>
+      </c>
+      <c r="E126" s="16" t="s">
+        <v>502</v>
       </c>
       <c r="F126" s="2" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
       <c r="G126" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H126" s="2" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
       <c r="I126" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="J126" s="2" t="s">
-        <v>458</v>
+        <v>464</v>
+      </c>
+      <c r="J126" s="16" t="s">
+        <v>502</v>
       </c>
       <c r="K126" s="2" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="L126" s="1" t="s">
-        <v>478</v>
+        <v>472</v>
       </c>
       <c r="M126" s="1" t="s">
         <v>19</v>
@@ -6757,37 +6758,37 @@
         <v>14</v>
       </c>
       <c r="D127" s="1" t="s">
-        <v>470</v>
-      </c>
-      <c r="E127" s="2" t="s">
-        <v>458</v>
+        <v>464</v>
+      </c>
+      <c r="E127" s="16" t="s">
+        <v>502</v>
       </c>
       <c r="F127" s="2" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="G127" s="2" t="s">
-        <v>478</v>
+        <v>472</v>
       </c>
       <c r="H127" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="I127" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="J127" s="16" t="s">
+        <v>502</v>
+      </c>
+      <c r="K127" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="L127" s="1" t="s">
         <v>473</v>
       </c>
-      <c r="I127" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="J127" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="K127" s="2" t="s">
-        <v>475</v>
-      </c>
-      <c r="L127" s="1" t="s">
-        <v>479</v>
-      </c>
       <c r="M127" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="128" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>188</v>
       </c>
@@ -6798,16 +6799,16 @@
         <v>14</v>
       </c>
       <c r="D128" s="1" t="s">
-        <v>480</v>
-      </c>
-      <c r="E128" s="2" t="s">
-        <v>393</v>
+        <v>474</v>
+      </c>
+      <c r="E128" s="16" t="s">
+        <v>503</v>
       </c>
       <c r="F128" s="2" t="s">
-        <v>481</v>
+        <v>475</v>
       </c>
       <c r="G128" s="2" t="s">
-        <v>482</v>
+        <v>476</v>
       </c>
       <c r="H128" s="2" t="s">
         <v>230</v>
@@ -6828,7 +6829,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="129" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>188</v>
       </c>
@@ -6839,16 +6840,16 @@
         <v>14</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>480</v>
-      </c>
-      <c r="E129" s="2" t="s">
-        <v>439</v>
+        <v>474</v>
+      </c>
+      <c r="E129" s="16" t="s">
+        <v>504</v>
       </c>
       <c r="F129" s="2" t="s">
-        <v>483</v>
+        <v>477</v>
       </c>
       <c r="G129" s="2" t="s">
-        <v>484</v>
+        <v>478</v>
       </c>
       <c r="H129" s="2" t="s">
         <v>230</v>
@@ -6869,7 +6870,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="130" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>188</v>
       </c>
@@ -6880,16 +6881,16 @@
         <v>14</v>
       </c>
       <c r="D130" s="1" t="s">
-        <v>485</v>
-      </c>
-      <c r="E130" s="2" t="s">
-        <v>393</v>
+        <v>479</v>
+      </c>
+      <c r="E130" s="16" t="s">
+        <v>505</v>
       </c>
       <c r="F130" s="2" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="G130" s="2" t="s">
-        <v>487</v>
+        <v>481</v>
       </c>
       <c r="H130" s="2" t="s">
         <v>230</v>
@@ -6907,17 +6908,17 @@
         <v>361</v>
       </c>
       <c r="M130" s="1" t="s">
-        <v>488</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M93" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:M130" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="ERROR">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="ERROR">
       <formula>NOT(ISERROR(SEARCH("ERROR",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="REVISAR">
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="REVISAR">
       <formula>NOT(ISERROR(SEARCH("REVISAR",C1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>